<commit_message>
error corrects: unit & ww-> lw conversions
</commit_message>
<xml_diff>
--- a/modified_data/Stokcholm_stad_contaminated.xlsx
+++ b/modified_data/Stokcholm_stad_contaminated.xlsx
@@ -974,7 +974,7 @@
         <v>49</v>
       </c>
       <c r="K2" t="n">
-        <v>0.35257406767628</v>
+        <v>35.257406767628</v>
       </c>
       <c r="L2" t="s">
         <v>50</v>
@@ -1051,7 +1051,7 @@
         <v>55</v>
       </c>
       <c r="K3" t="n">
-        <v>2.05747012284303</v>
+        <v>205.747012284303</v>
       </c>
       <c r="L3" t="s">
         <v>50</v>
@@ -1128,7 +1128,7 @@
         <v>58</v>
       </c>
       <c r="K4" t="n">
-        <v>7.86437243790351</v>
+        <v>786.437243790351</v>
       </c>
       <c r="L4" t="s">
         <v>50</v>
@@ -1205,7 +1205,7 @@
         <v>61</v>
       </c>
       <c r="K5" t="n">
-        <v>5.85384086256571</v>
+        <v>585.384086256572</v>
       </c>
       <c r="L5" t="s">
         <v>50</v>
@@ -1282,7 +1282,7 @@
         <v>64</v>
       </c>
       <c r="K6" t="n">
-        <v>14.7562541015018</v>
+        <v>1475.62541015018</v>
       </c>
       <c r="L6" t="s">
         <v>50</v>
@@ -1359,7 +1359,7 @@
         <v>67</v>
       </c>
       <c r="K7" t="n">
-        <v>13.5953016075994</v>
+        <v>1359.53016075994</v>
       </c>
       <c r="L7" t="s">
         <v>50</v>
@@ -1436,7 +1436,7 @@
         <v>70</v>
       </c>
       <c r="K8" t="n">
-        <v>3.57166107195083</v>
+        <v>357.166107195083</v>
       </c>
       <c r="L8" t="s">
         <v>50</v>
@@ -1513,7 +1513,7 @@
         <v>74</v>
       </c>
       <c r="K9" t="n">
-        <v>0.0728553694738795</v>
+        <v>7.28553694738795</v>
       </c>
       <c r="L9" t="s">
         <v>50</v>
@@ -1590,7 +1590,7 @@
         <v>77</v>
       </c>
       <c r="K10" t="n">
-        <v>0.0506997815756782</v>
+        <v>5.06997815756782</v>
       </c>
       <c r="L10" t="s">
         <v>50</v>
@@ -1667,7 +1667,7 @@
         <v>80</v>
       </c>
       <c r="K11" t="n">
-        <v>0.0301569294860732</v>
+        <v>3.01569294860732</v>
       </c>
       <c r="L11" t="s">
         <v>50</v>
@@ -2745,7 +2745,7 @@
         <v>49</v>
       </c>
       <c r="K25" t="n">
-        <v>0.627088504560102</v>
+        <v>62.7088504560102</v>
       </c>
       <c r="L25" t="s">
         <v>50</v>
@@ -2822,7 +2822,7 @@
         <v>55</v>
       </c>
       <c r="K26" t="n">
-        <v>3.73116282555749</v>
+        <v>373.116282555749</v>
       </c>
       <c r="L26" t="s">
         <v>50</v>
@@ -2899,7 +2899,7 @@
         <v>58</v>
       </c>
       <c r="K27" t="n">
-        <v>14.869947701653</v>
+        <v>1486.9947701653</v>
       </c>
       <c r="L27" t="s">
         <v>50</v>
@@ -2976,7 +2976,7 @@
         <v>61</v>
       </c>
       <c r="K28" t="n">
-        <v>10.0743007089604</v>
+        <v>1007.43007089604</v>
       </c>
       <c r="L28" t="s">
         <v>50</v>
@@ -3053,7 +3053,7 @@
         <v>64</v>
       </c>
       <c r="K29" t="n">
-        <v>21.3314369626699</v>
+        <v>2133.14369626699</v>
       </c>
       <c r="L29" t="s">
         <v>50</v>
@@ -3130,7 +3130,7 @@
         <v>67</v>
       </c>
       <c r="K30" t="n">
-        <v>19.7780327420251</v>
+        <v>1977.80327420251</v>
       </c>
       <c r="L30" t="s">
         <v>50</v>
@@ -3207,7 +3207,7 @@
         <v>70</v>
       </c>
       <c r="K31" t="n">
-        <v>5.01944215677312</v>
+        <v>501.944215677312</v>
       </c>
       <c r="L31" t="s">
         <v>50</v>
@@ -3284,7 +3284,7 @@
         <v>74</v>
       </c>
       <c r="K32" t="n">
-        <v>0.0735972148178375</v>
+        <v>7.35972148178375</v>
       </c>
       <c r="L32" t="s">
         <v>50</v>
@@ -3361,7 +3361,7 @@
         <v>77</v>
       </c>
       <c r="K33" t="n">
-        <v>0.0318791805609367</v>
+        <v>3.18791805609367</v>
       </c>
       <c r="L33" t="s">
         <v>50</v>
@@ -3438,7 +3438,7 @@
         <v>80</v>
       </c>
       <c r="K34" t="n">
-        <v>0.0439997421041557</v>
+        <v>4.39997421041557</v>
       </c>
       <c r="L34" t="s">
         <v>50</v>
@@ -3515,7 +3515,7 @@
         <v>125</v>
       </c>
       <c r="K35" t="n">
-        <v>0.514853267108331</v>
+        <v>51.4853267108331</v>
       </c>
       <c r="L35" t="s">
         <v>50</v>
@@ -3592,7 +3592,7 @@
         <v>128</v>
       </c>
       <c r="K36" t="n">
-        <v>0.0190752578532495</v>
+        <v>1.90752578532495</v>
       </c>
       <c r="L36" t="s">
         <v>50</v>
@@ -4593,7 +4593,7 @@
         <v>49</v>
       </c>
       <c r="K49" t="n">
-        <v>0.233434250136836</v>
+        <v>23.3434250136836</v>
       </c>
       <c r="L49" t="s">
         <v>50</v>
@@ -4670,7 +4670,7 @@
         <v>55</v>
       </c>
       <c r="K50" t="n">
-        <v>1.7616824028462</v>
+        <v>176.16824028462</v>
       </c>
       <c r="L50" t="s">
         <v>50</v>
@@ -4747,7 +4747,7 @@
         <v>58</v>
       </c>
       <c r="K51" t="n">
-        <v>8.49765097609925</v>
+        <v>849.765097609925</v>
       </c>
       <c r="L51" t="s">
         <v>50</v>
@@ -4824,7 +4824,7 @@
         <v>61</v>
       </c>
       <c r="K52" t="n">
-        <v>7.11137053001277</v>
+        <v>711.137053001277</v>
       </c>
       <c r="L52" t="s">
         <v>50</v>
@@ -4901,7 +4901,7 @@
         <v>64</v>
       </c>
       <c r="K53" t="n">
-        <v>17.2208110974275</v>
+        <v>1722.08110974275</v>
       </c>
       <c r="L53" t="s">
         <v>50</v>
@@ -4978,7 +4978,7 @@
         <v>67</v>
       </c>
       <c r="K54" t="n">
-        <v>15.962857484948</v>
+        <v>1596.2857484948</v>
       </c>
       <c r="L54" t="s">
         <v>50</v>
@@ -5055,7 +5055,7 @@
         <v>70</v>
       </c>
       <c r="K55" t="n">
-        <v>5.55894795657727</v>
+        <v>555.894795657727</v>
       </c>
       <c r="L55" t="s">
         <v>50</v>
@@ -5132,7 +5132,7 @@
         <v>74</v>
       </c>
       <c r="K56" t="n">
-        <v>0.0986111111111111</v>
+        <v>9.86111111111111</v>
       </c>
       <c r="L56" t="s">
         <v>50</v>
@@ -5209,7 +5209,7 @@
         <v>77</v>
       </c>
       <c r="K57" t="n">
-        <v>0.0208333333333333</v>
+        <v>2.08333333333333</v>
       </c>
       <c r="L57" t="s">
         <v>50</v>
@@ -5286,7 +5286,7 @@
         <v>80</v>
       </c>
       <c r="K58" t="n">
-        <v>0.0472222222222222</v>
+        <v>4.72222222222222</v>
       </c>
       <c r="L58" t="s">
         <v>50</v>
@@ -5363,7 +5363,7 @@
         <v>132</v>
       </c>
       <c r="K59" t="n">
-        <v>0.0166666666666667</v>
+        <v>1.66666666666667</v>
       </c>
       <c r="L59" t="s">
         <v>50</v>
@@ -5440,7 +5440,7 @@
         <v>135</v>
       </c>
       <c r="K60" t="n">
-        <v>0.0166666666666667</v>
+        <v>1.66666666666667</v>
       </c>
       <c r="L60" t="s">
         <v>50</v>
@@ -5517,7 +5517,7 @@
         <v>128</v>
       </c>
       <c r="K61" t="n">
-        <v>0.0285075716110199</v>
+        <v>2.85075716110199</v>
       </c>
       <c r="L61" t="s">
         <v>50</v>
@@ -6441,7 +6441,7 @@
         <v>49</v>
       </c>
       <c r="K73" t="n">
-        <v>0.162518996711452</v>
+        <v>16.2518996711452</v>
       </c>
       <c r="L73" t="s">
         <v>50</v>
@@ -6518,7 +6518,7 @@
         <v>55</v>
       </c>
       <c r="K74" t="n">
-        <v>0.972374679172541</v>
+        <v>97.2374679172541</v>
       </c>
       <c r="L74" t="s">
         <v>50</v>
@@ -6595,7 +6595,7 @@
         <v>58</v>
       </c>
       <c r="K75" t="n">
-        <v>3.72952525906693</v>
+        <v>372.952525906693</v>
       </c>
       <c r="L75" t="s">
         <v>50</v>
@@ -6672,7 +6672,7 @@
         <v>61</v>
       </c>
       <c r="K76" t="n">
-        <v>2.94701576528738</v>
+        <v>294.701576528738</v>
       </c>
       <c r="L76" t="s">
         <v>50</v>
@@ -6749,7 +6749,7 @@
         <v>64</v>
       </c>
       <c r="K77" t="n">
-        <v>6.13424956466535</v>
+        <v>613.424956466535</v>
       </c>
       <c r="L77" t="s">
         <v>50</v>
@@ -6826,7 +6826,7 @@
         <v>67</v>
       </c>
       <c r="K78" t="n">
-        <v>5.80951719960614</v>
+        <v>580.951719960614</v>
       </c>
       <c r="L78" t="s">
         <v>50</v>
@@ -6903,7 +6903,7 @@
         <v>70</v>
       </c>
       <c r="K79" t="n">
-        <v>1.9039739240098</v>
+        <v>190.39739240098</v>
       </c>
       <c r="L79" t="s">
         <v>50</v>
@@ -6980,7 +6980,7 @@
         <v>139</v>
       </c>
       <c r="K80" t="n">
-        <v>0.0423842676494724</v>
+        <v>4.23842676494724</v>
       </c>
       <c r="L80" t="s">
         <v>50</v>
@@ -7057,7 +7057,7 @@
         <v>74</v>
       </c>
       <c r="K81" t="n">
-        <v>0.0597232862333474</v>
+        <v>5.97232862333474</v>
       </c>
       <c r="L81" t="s">
         <v>50</v>
@@ -7134,7 +7134,7 @@
         <v>77</v>
       </c>
       <c r="K82" t="n">
-        <v>0.0179972591041888</v>
+        <v>1.79972591041888</v>
       </c>
       <c r="L82" t="s">
         <v>50</v>
@@ -7211,7 +7211,7 @@
         <v>80</v>
       </c>
       <c r="K83" t="n">
-        <v>0.0393820486909681</v>
+        <v>3.93820486909681</v>
       </c>
       <c r="L83" t="s">
         <v>50</v>
@@ -7288,7 +7288,7 @@
         <v>132</v>
       </c>
       <c r="K84" t="n">
-        <v>0.0147381657962937</v>
+        <v>1.47381657962937</v>
       </c>
       <c r="L84" t="s">
         <v>50</v>
@@ -7365,7 +7365,7 @@
         <v>135</v>
       </c>
       <c r="K85" t="n">
-        <v>0.0170981988813212</v>
+        <v>1.70981988813212</v>
       </c>
       <c r="L85" t="s">
         <v>50</v>
@@ -7442,7 +7442,7 @@
         <v>128</v>
       </c>
       <c r="K86" t="n">
-        <v>0.0251377009921314</v>
+        <v>2.51377009921314</v>
       </c>
       <c r="L86" t="s">
         <v>50</v>
@@ -8366,7 +8366,7 @@
         <v>49</v>
       </c>
       <c r="K98" t="n">
-        <v>0.671267194431348</v>
+        <v>67.1267194431348</v>
       </c>
       <c r="L98" t="s">
         <v>50</v>
@@ -8443,7 +8443,7 @@
         <v>55</v>
       </c>
       <c r="K99" t="n">
-        <v>4.27842689436243</v>
+        <v>427.842689436243</v>
       </c>
       <c r="L99" t="s">
         <v>50</v>
@@ -8520,7 +8520,7 @@
         <v>58</v>
       </c>
       <c r="K100" t="n">
-        <v>19.1970684711632</v>
+        <v>1919.70684711632</v>
       </c>
       <c r="L100" t="s">
         <v>50</v>
@@ -8597,7 +8597,7 @@
         <v>61</v>
       </c>
       <c r="K101" t="n">
-        <v>15.0788441230553</v>
+        <v>1507.88441230553</v>
       </c>
       <c r="L101" t="s">
         <v>50</v>
@@ -8674,7 +8674,7 @@
         <v>64</v>
       </c>
       <c r="K102" t="n">
-        <v>32.051051213615</v>
+        <v>3205.1051213615</v>
       </c>
       <c r="L102" t="s">
         <v>50</v>
@@ -8751,7 +8751,7 @@
         <v>67</v>
       </c>
       <c r="K103" t="n">
-        <v>29.0744243877777</v>
+        <v>2907.44243877777</v>
       </c>
       <c r="L103" t="s">
         <v>50</v>
@@ -8828,7 +8828,7 @@
         <v>70</v>
       </c>
       <c r="K104" t="n">
-        <v>10.6306210552879</v>
+        <v>1063.06210552879</v>
       </c>
       <c r="L104" t="s">
         <v>50</v>
@@ -8905,7 +8905,7 @@
         <v>74</v>
       </c>
       <c r="K105" t="n">
-        <v>0.339330296176622</v>
+        <v>33.9330296176622</v>
       </c>
       <c r="L105" t="s">
         <v>50</v>
@@ -8982,7 +8982,7 @@
         <v>77</v>
       </c>
       <c r="K106" t="n">
-        <v>0.047110516549102</v>
+        <v>4.7110516549102</v>
       </c>
       <c r="L106" t="s">
         <v>50</v>
@@ -9059,7 +9059,7 @@
         <v>80</v>
       </c>
       <c r="K107" t="n">
-        <v>0.104171326299452</v>
+        <v>10.4171326299452</v>
       </c>
       <c r="L107" t="s">
         <v>50</v>
@@ -9136,7 +9136,7 @@
         <v>132</v>
       </c>
       <c r="K108" t="n">
-        <v>0.0448186971427221</v>
+        <v>4.48186971427221</v>
       </c>
       <c r="L108" t="s">
         <v>50</v>
@@ -9213,7 +9213,7 @@
         <v>135</v>
       </c>
       <c r="K109" t="n">
-        <v>0.0697536895079866</v>
+        <v>6.97536895079866</v>
       </c>
       <c r="L109" t="s">
         <v>50</v>
@@ -9290,7 +9290,7 @@
         <v>128</v>
       </c>
       <c r="K110" t="n">
-        <v>0.0215206008583668</v>
+        <v>2.15206008583668</v>
       </c>
       <c r="L110" t="s">
         <v>50</v>
@@ -10137,7 +10137,7 @@
         <v>49</v>
       </c>
       <c r="K121" t="n">
-        <v>1.92725373663352</v>
+        <v>192.725373663352</v>
       </c>
       <c r="L121" t="s">
         <v>50</v>
@@ -10214,7 +10214,7 @@
         <v>55</v>
       </c>
       <c r="K122" t="n">
-        <v>7.56215876444345</v>
+        <v>756.215876444345</v>
       </c>
       <c r="L122" t="s">
         <v>50</v>
@@ -10291,7 +10291,7 @@
         <v>58</v>
       </c>
       <c r="K123" t="n">
-        <v>36.0037936536155</v>
+        <v>3600.37936536155</v>
       </c>
       <c r="L123" t="s">
         <v>50</v>
@@ -10368,7 +10368,7 @@
         <v>61</v>
       </c>
       <c r="K124" t="n">
-        <v>33.4221481194205</v>
+        <v>3342.21481194205</v>
       </c>
       <c r="L124" t="s">
         <v>50</v>
@@ -10445,7 +10445,7 @@
         <v>64</v>
       </c>
       <c r="K125" t="n">
-        <v>72.1165713361096</v>
+        <v>7211.65713361096</v>
       </c>
       <c r="L125" t="s">
         <v>50</v>
@@ -10522,7 +10522,7 @@
         <v>67</v>
       </c>
       <c r="K126" t="n">
-        <v>65.1357690866383</v>
+        <v>6513.57690866384</v>
       </c>
       <c r="L126" t="s">
         <v>50</v>
@@ -10599,7 +10599,7 @@
         <v>70</v>
       </c>
       <c r="K127" t="n">
-        <v>25.0184581908998</v>
+        <v>2501.84581908998</v>
       </c>
       <c r="L127" t="s">
         <v>50</v>
@@ -10676,7 +10676,7 @@
         <v>74</v>
       </c>
       <c r="K128" t="n">
-        <v>0.618883860265159</v>
+        <v>61.8883860265159</v>
       </c>
       <c r="L128" t="s">
         <v>50</v>
@@ -10753,7 +10753,7 @@
         <v>77</v>
       </c>
       <c r="K129" t="n">
-        <v>0.200031526701989</v>
+        <v>20.0031526701989</v>
       </c>
       <c r="L129" t="s">
         <v>50</v>
@@ -10830,7 +10830,7 @@
         <v>80</v>
       </c>
       <c r="K130" t="n">
-        <v>0.174802964676868</v>
+        <v>17.4802964676868</v>
       </c>
       <c r="L130" t="s">
         <v>50</v>
@@ -10907,7 +10907,7 @@
         <v>135</v>
       </c>
       <c r="K131" t="n">
-        <v>0.206920376861473</v>
+        <v>20.6920376861473</v>
       </c>
       <c r="L131" t="s">
         <v>50</v>
@@ -10984,7 +10984,7 @@
         <v>128</v>
       </c>
       <c r="K132" t="n">
-        <v>0.188198594835213</v>
+        <v>18.8198594835213</v>
       </c>
       <c r="L132" t="s">
         <v>50</v>
@@ -12370,7 +12370,7 @@
         <v>49</v>
       </c>
       <c r="K150" t="n">
-        <v>0.864881629077504</v>
+        <v>86.4881629077504</v>
       </c>
       <c r="L150" t="s">
         <v>50</v>
@@ -12447,7 +12447,7 @@
         <v>55</v>
       </c>
       <c r="K151" t="n">
-        <v>3.36718709038976</v>
+        <v>336.718709038976</v>
       </c>
       <c r="L151" t="s">
         <v>50</v>
@@ -12524,7 +12524,7 @@
         <v>58</v>
       </c>
       <c r="K152" t="n">
-        <v>9.11728401790868</v>
+        <v>911.728401790868</v>
       </c>
       <c r="L152" t="s">
         <v>50</v>
@@ -12601,7 +12601,7 @@
         <v>61</v>
       </c>
       <c r="K153" t="n">
-        <v>7.80837167329407</v>
+        <v>780.837167329407</v>
       </c>
       <c r="L153" t="s">
         <v>50</v>
@@ -12678,7 +12678,7 @@
         <v>64</v>
       </c>
       <c r="K154" t="n">
-        <v>13.7127910791911</v>
+        <v>1371.27910791911</v>
       </c>
       <c r="L154" t="s">
         <v>50</v>
@@ -12755,7 +12755,7 @@
         <v>67</v>
       </c>
       <c r="K155" t="n">
-        <v>12.8961941563068</v>
+        <v>1289.61941563068</v>
       </c>
       <c r="L155" t="s">
         <v>50</v>
@@ -12832,7 +12832,7 @@
         <v>70</v>
       </c>
       <c r="K156" t="n">
-        <v>5.2117885879285</v>
+        <v>521.17885879285</v>
       </c>
       <c r="L156" t="s">
         <v>50</v>
@@ -12909,7 +12909,7 @@
         <v>74</v>
       </c>
       <c r="K157" t="n">
-        <v>0.268055477021007</v>
+        <v>26.8055477021007</v>
       </c>
       <c r="L157" t="s">
         <v>50</v>
@@ -12986,7 +12986,7 @@
         <v>77</v>
       </c>
       <c r="K158" t="n">
-        <v>0.104076806156134</v>
+        <v>10.4076806156134</v>
       </c>
       <c r="L158" t="s">
         <v>50</v>
@@ -13063,7 +13063,7 @@
         <v>80</v>
       </c>
       <c r="K159" t="n">
-        <v>0.127801379813179</v>
+        <v>12.7801379813179</v>
       </c>
       <c r="L159" t="s">
         <v>50</v>
@@ -13140,7 +13140,7 @@
         <v>128</v>
       </c>
       <c r="K160" t="n">
-        <v>0.0807285714285661</v>
+        <v>8.07285714285661</v>
       </c>
       <c r="L160" t="s">
         <v>50</v>
@@ -14449,7 +14449,7 @@
         <v>49</v>
       </c>
       <c r="K177" t="n">
-        <v>0.422037676524976</v>
+        <v>42.2037676524976</v>
       </c>
       <c r="L177" t="s">
         <v>50</v>
@@ -14526,7 +14526,7 @@
         <v>55</v>
       </c>
       <c r="K178" t="n">
-        <v>2.50223497674</v>
+        <v>250.223497674</v>
       </c>
       <c r="L178" t="s">
         <v>50</v>
@@ -14603,7 +14603,7 @@
         <v>58</v>
       </c>
       <c r="K179" t="n">
-        <v>9.05974085472145</v>
+        <v>905.974085472145</v>
       </c>
       <c r="L179" t="s">
         <v>50</v>
@@ -14680,7 +14680,7 @@
         <v>61</v>
       </c>
       <c r="K180" t="n">
-        <v>6.6735380369045</v>
+        <v>667.353803690449</v>
       </c>
       <c r="L180" t="s">
         <v>50</v>
@@ -14757,7 +14757,7 @@
         <v>64</v>
       </c>
       <c r="K181" t="n">
-        <v>13.8134328648587</v>
+        <v>1381.34328648587</v>
       </c>
       <c r="L181" t="s">
         <v>50</v>
@@ -14834,7 +14834,7 @@
         <v>67</v>
       </c>
       <c r="K182" t="n">
-        <v>12.0950260370052</v>
+        <v>1209.50260370052</v>
       </c>
       <c r="L182" t="s">
         <v>50</v>
@@ -14911,7 +14911,7 @@
         <v>70</v>
       </c>
       <c r="K183" t="n">
-        <v>4.97943001646247</v>
+        <v>497.943001646247</v>
       </c>
       <c r="L183" t="s">
         <v>50</v>
@@ -14988,7 +14988,7 @@
         <v>74</v>
       </c>
       <c r="K184" t="n">
-        <v>0.0811441000688068</v>
+        <v>8.11441000688068</v>
       </c>
       <c r="L184" t="s">
         <v>50</v>
@@ -15065,7 +15065,7 @@
         <v>77</v>
       </c>
       <c r="K185" t="n">
-        <v>0.0247290624601665</v>
+        <v>2.47290624601665</v>
       </c>
       <c r="L185" t="s">
         <v>50</v>
@@ -15142,7 +15142,7 @@
         <v>80</v>
       </c>
       <c r="K186" t="n">
-        <v>0.025238942660708</v>
+        <v>2.5238942660708</v>
       </c>
       <c r="L186" t="s">
         <v>50</v>
@@ -15219,7 +15219,7 @@
         <v>132</v>
       </c>
       <c r="K187" t="n">
-        <v>0.0282084350170438</v>
+        <v>2.82084350170438</v>
       </c>
       <c r="L187" t="s">
         <v>50</v>
@@ -15296,7 +15296,7 @@
         <v>135</v>
       </c>
       <c r="K188" t="n">
-        <v>0.0460922726838815</v>
+        <v>4.60922726838815</v>
       </c>
       <c r="L188" t="s">
         <v>50</v>
@@ -15373,7 +15373,7 @@
         <v>128</v>
       </c>
       <c r="K189" t="n">
-        <v>0.139542857142856</v>
+        <v>13.9542857142856</v>
       </c>
       <c r="L189" t="s">
         <v>50</v>
@@ -18810,7 +18810,7 @@
         <v>49</v>
       </c>
       <c r="K234" t="n">
-        <v>0.317712660701218</v>
+        <v>31.7712660701218</v>
       </c>
       <c r="L234" t="s">
         <v>50</v>
@@ -18887,7 +18887,7 @@
         <v>55</v>
       </c>
       <c r="K235" t="n">
-        <v>0.644984637123296</v>
+        <v>64.4984637123296</v>
       </c>
       <c r="L235" t="s">
         <v>50</v>
@@ -18964,7 +18964,7 @@
         <v>58</v>
       </c>
       <c r="K236" t="n">
-        <v>2.29883355651903</v>
+        <v>229.883355651904</v>
       </c>
       <c r="L236" t="s">
         <v>50</v>
@@ -19041,7 +19041,7 @@
         <v>61</v>
       </c>
       <c r="K237" t="n">
-        <v>1.85834843607259</v>
+        <v>185.834843607259</v>
       </c>
       <c r="L237" t="s">
         <v>50</v>
@@ -19118,7 +19118,7 @@
         <v>64</v>
       </c>
       <c r="K238" t="n">
-        <v>4.11921390374294</v>
+        <v>411.921390374294</v>
       </c>
       <c r="L238" t="s">
         <v>50</v>
@@ -19195,7 +19195,7 @@
         <v>67</v>
       </c>
       <c r="K239" t="n">
-        <v>3.88375937306894</v>
+        <v>388.375937306894</v>
       </c>
       <c r="L239" t="s">
         <v>50</v>
@@ -19272,7 +19272,7 @@
         <v>70</v>
       </c>
       <c r="K240" t="n">
-        <v>1.05144470458157</v>
+        <v>105.144470458157</v>
       </c>
       <c r="L240" t="s">
         <v>50</v>
@@ -19349,7 +19349,7 @@
         <v>74</v>
       </c>
       <c r="K241" t="n">
-        <v>0.028964297355877</v>
+        <v>2.8964297355877</v>
       </c>
       <c r="L241" t="s">
         <v>50</v>
@@ -19426,7 +19426,7 @@
         <v>77</v>
       </c>
       <c r="K242" t="n">
-        <v>0.0295103905478816</v>
+        <v>2.95103905478816</v>
       </c>
       <c r="L242" t="s">
         <v>50</v>
@@ -19503,7 +19503,7 @@
         <v>80</v>
       </c>
       <c r="K243" t="n">
-        <v>0.0178443389113027</v>
+        <v>1.78443389113027</v>
       </c>
       <c r="L243" t="s">
         <v>50</v>
@@ -20581,7 +20581,7 @@
         <v>49</v>
       </c>
       <c r="K257" t="n">
-        <v>0.630837210006851</v>
+        <v>63.0837210006851</v>
       </c>
       <c r="L257" t="s">
         <v>50</v>
@@ -20658,7 +20658,7 @@
         <v>55</v>
       </c>
       <c r="K258" t="n">
-        <v>2.16576211297989</v>
+        <v>216.576211297989</v>
       </c>
       <c r="L258" t="s">
         <v>50</v>
@@ -20735,7 +20735,7 @@
         <v>58</v>
       </c>
       <c r="K259" t="n">
-        <v>10.8856083877779</v>
+        <v>1088.56083877778</v>
       </c>
       <c r="L259" t="s">
         <v>50</v>
@@ -20812,7 +20812,7 @@
         <v>61</v>
       </c>
       <c r="K260" t="n">
-        <v>8.47695061863842</v>
+        <v>847.695061863842</v>
       </c>
       <c r="L260" t="s">
         <v>50</v>
@@ -20889,7 +20889,7 @@
         <v>64</v>
       </c>
       <c r="K261" t="n">
-        <v>22.2266066820551</v>
+        <v>2222.66066820551</v>
       </c>
       <c r="L261" t="s">
         <v>50</v>
@@ -20966,7 +20966,7 @@
         <v>67</v>
       </c>
       <c r="K262" t="n">
-        <v>18.5460336438459</v>
+        <v>1854.60336438459</v>
       </c>
       <c r="L262" t="s">
         <v>50</v>
@@ -21043,7 +21043,7 @@
         <v>70</v>
       </c>
       <c r="K263" t="n">
-        <v>5.38094831036423</v>
+        <v>538.094831036423</v>
       </c>
       <c r="L263" t="s">
         <v>50</v>
@@ -21120,7 +21120,7 @@
         <v>74</v>
       </c>
       <c r="K264" t="n">
-        <v>0.137764799999998</v>
+        <v>13.7764799999998</v>
       </c>
       <c r="L264" t="s">
         <v>50</v>
@@ -21197,7 +21197,7 @@
         <v>77</v>
       </c>
       <c r="K265" t="n">
-        <v>0.0440081999999994</v>
+        <v>4.40081999999994</v>
       </c>
       <c r="L265" t="s">
         <v>50</v>
@@ -21274,7 +21274,7 @@
         <v>80</v>
       </c>
       <c r="K266" t="n">
-        <v>0.0631421999999991</v>
+        <v>6.31421999999991</v>
       </c>
       <c r="L266" t="s">
         <v>50</v>
@@ -21351,7 +21351,7 @@
         <v>132</v>
       </c>
       <c r="K267" t="n">
-        <v>0.0210473999999997</v>
+        <v>2.10473999999997</v>
       </c>
       <c r="L267" t="s">
         <v>50</v>
@@ -21428,7 +21428,7 @@
         <v>128</v>
       </c>
       <c r="K268" t="n">
-        <v>0.00191339999999997</v>
+        <v>0.191339999999997</v>
       </c>
       <c r="L268" t="s">
         <v>50</v>
@@ -22429,7 +22429,7 @@
         <v>49</v>
       </c>
       <c r="K281" t="n">
-        <v>0.263460186217933</v>
+        <v>26.3460186217933</v>
       </c>
       <c r="L281" t="s">
         <v>50</v>
@@ -22506,7 +22506,7 @@
         <v>55</v>
       </c>
       <c r="K282" t="n">
-        <v>0.778984409097522</v>
+        <v>77.8984409097522</v>
       </c>
       <c r="L282" t="s">
         <v>50</v>
@@ -22583,7 +22583,7 @@
         <v>58</v>
       </c>
       <c r="K283" t="n">
-        <v>3.10648125697105</v>
+        <v>310.648125697105</v>
       </c>
       <c r="L283" t="s">
         <v>50</v>
@@ -22660,7 +22660,7 @@
         <v>61</v>
       </c>
       <c r="K284" t="n">
-        <v>2.55729899131953</v>
+        <v>255.729899131953</v>
       </c>
       <c r="L284" t="s">
         <v>50</v>
@@ -22737,7 +22737,7 @@
         <v>64</v>
       </c>
       <c r="K285" t="n">
-        <v>6.14241852965424</v>
+        <v>614.241852965424</v>
       </c>
       <c r="L285" t="s">
         <v>50</v>
@@ -22814,7 +22814,7 @@
         <v>67</v>
       </c>
       <c r="K286" t="n">
-        <v>5.41658079142621</v>
+        <v>541.658079142622</v>
       </c>
       <c r="L286" t="s">
         <v>50</v>
@@ -22891,7 +22891,7 @@
         <v>70</v>
       </c>
       <c r="K287" t="n">
-        <v>1.84847970515494</v>
+        <v>184.847970515494</v>
       </c>
       <c r="L287" t="s">
         <v>50</v>
@@ -22968,7 +22968,7 @@
         <v>74</v>
       </c>
       <c r="K288" t="n">
-        <v>0.0544117647058823</v>
+        <v>5.44117647058823</v>
       </c>
       <c r="L288" t="s">
         <v>50</v>
@@ -23045,7 +23045,7 @@
         <v>77</v>
       </c>
       <c r="K289" t="n">
-        <v>0.00985294117647059</v>
+        <v>0.985294117647059</v>
       </c>
       <c r="L289" t="s">
         <v>50</v>
@@ -23122,7 +23122,7 @@
         <v>80</v>
       </c>
       <c r="K290" t="n">
-        <v>0.0279411764705882</v>
+        <v>2.79411764705882</v>
       </c>
       <c r="L290" t="s">
         <v>50</v>
@@ -23199,7 +23199,7 @@
         <v>128</v>
       </c>
       <c r="K291" t="n">
-        <v>0.0168214441588672</v>
+        <v>1.68214441588672</v>
       </c>
       <c r="L291" t="s">
         <v>50</v>
@@ -24123,7 +24123,7 @@
         <v>49</v>
       </c>
       <c r="K303" t="n">
-        <v>0.284143918581415</v>
+        <v>28.4143918581415</v>
       </c>
       <c r="L303" t="s">
         <v>50</v>
@@ -24200,7 +24200,7 @@
         <v>55</v>
       </c>
       <c r="K304" t="n">
-        <v>0.855092256260678</v>
+        <v>85.5092256260678</v>
       </c>
       <c r="L304" t="s">
         <v>50</v>
@@ -24277,7 +24277,7 @@
         <v>58</v>
       </c>
       <c r="K305" t="n">
-        <v>3.61546007911576</v>
+        <v>361.546007911576</v>
       </c>
       <c r="L305" t="s">
         <v>50</v>
@@ -24354,7 +24354,7 @@
         <v>61</v>
       </c>
       <c r="K306" t="n">
-        <v>3.17269613437406</v>
+        <v>317.269613437406</v>
       </c>
       <c r="L306" t="s">
         <v>50</v>
@@ -24431,7 +24431,7 @@
         <v>64</v>
       </c>
       <c r="K307" t="n">
-        <v>6.97435429824405</v>
+        <v>697.435429824405</v>
       </c>
       <c r="L307" t="s">
         <v>50</v>
@@ -24508,7 +24508,7 @@
         <v>67</v>
       </c>
       <c r="K308" t="n">
-        <v>6.4807821839177</v>
+        <v>648.07821839177</v>
       </c>
       <c r="L308" t="s">
         <v>50</v>
@@ -24585,7 +24585,7 @@
         <v>70</v>
       </c>
       <c r="K309" t="n">
-        <v>2.3506261090604</v>
+        <v>235.06261090604</v>
       </c>
       <c r="L309" t="s">
         <v>50</v>
@@ -24662,7 +24662,7 @@
         <v>139</v>
       </c>
       <c r="K310" t="n">
-        <v>0.0102320879120878</v>
+        <v>1.02320879120878</v>
       </c>
       <c r="L310" t="s">
         <v>50</v>
@@ -24739,7 +24739,7 @@
         <v>74</v>
       </c>
       <c r="K311" t="n">
-        <v>0.0894511530500539</v>
+        <v>8.94511530500539</v>
       </c>
       <c r="L311" t="s">
         <v>50</v>
@@ -24816,7 +24816,7 @@
         <v>77</v>
       </c>
       <c r="K312" t="n">
-        <v>0.0258459666933215</v>
+        <v>2.58459666933215</v>
       </c>
       <c r="L312" t="s">
         <v>50</v>
@@ -24893,7 +24893,7 @@
         <v>80</v>
       </c>
       <c r="K313" t="n">
-        <v>0.0339707739094534</v>
+        <v>3.39707739094534</v>
       </c>
       <c r="L313" t="s">
         <v>50</v>
@@ -24970,7 +24970,7 @@
         <v>132</v>
       </c>
       <c r="K314" t="n">
-        <v>0.0147467599182973</v>
+        <v>1.47467599182973</v>
       </c>
       <c r="L314" t="s">
         <v>50</v>
@@ -25047,7 +25047,7 @@
         <v>135</v>
       </c>
       <c r="K315" t="n">
-        <v>0.0372113039551939</v>
+        <v>3.72113039551939</v>
       </c>
       <c r="L315" t="s">
         <v>50</v>
@@ -25124,7 +25124,7 @@
         <v>128</v>
       </c>
       <c r="K316" t="n">
-        <v>0.0247574353612486</v>
+        <v>2.47574353612486</v>
       </c>
       <c r="L316" t="s">
         <v>50</v>
@@ -26048,7 +26048,7 @@
         <v>49</v>
       </c>
       <c r="K328" t="n">
-        <v>0.751814503164994</v>
+        <v>75.1814503164994</v>
       </c>
       <c r="L328" t="s">
         <v>50</v>
@@ -26125,7 +26125,7 @@
         <v>55</v>
       </c>
       <c r="K329" t="n">
-        <v>2.05567608623733</v>
+        <v>205.567608623733</v>
       </c>
       <c r="L329" t="s">
         <v>50</v>
@@ -26202,7 +26202,7 @@
         <v>58</v>
       </c>
       <c r="K330" t="n">
-        <v>8.25376421203952</v>
+        <v>825.376421203952</v>
       </c>
       <c r="L330" t="s">
         <v>50</v>
@@ -26279,7 +26279,7 @@
         <v>61</v>
       </c>
       <c r="K331" t="n">
-        <v>6.36988409235937</v>
+        <v>636.988409235937</v>
       </c>
       <c r="L331" t="s">
         <v>50</v>
@@ -26356,7 +26356,7 @@
         <v>64</v>
       </c>
       <c r="K332" t="n">
-        <v>14.3161380438865</v>
+        <v>1431.61380438865</v>
       </c>
       <c r="L332" t="s">
         <v>50</v>
@@ -26433,7 +26433,7 @@
         <v>67</v>
       </c>
       <c r="K333" t="n">
-        <v>12.5846446124606</v>
+        <v>1258.46446124606</v>
       </c>
       <c r="L333" t="s">
         <v>50</v>
@@ -26510,7 +26510,7 @@
         <v>70</v>
       </c>
       <c r="K334" t="n">
-        <v>4.60507098136295</v>
+        <v>460.507098136295</v>
       </c>
       <c r="L334" t="s">
         <v>50</v>
@@ -26587,7 +26587,7 @@
         <v>74</v>
       </c>
       <c r="K335" t="n">
-        <v>0.282641309679191</v>
+        <v>28.2641309679191</v>
       </c>
       <c r="L335" t="s">
         <v>50</v>
@@ -26664,7 +26664,7 @@
         <v>80</v>
       </c>
       <c r="K336" t="n">
-        <v>0.0532280563492684</v>
+        <v>5.32280563492684</v>
       </c>
       <c r="L336" t="s">
         <v>50</v>
@@ -26741,7 +26741,7 @@
         <v>135</v>
       </c>
       <c r="K337" t="n">
-        <v>0.113410910627191</v>
+        <v>11.3410910627191</v>
       </c>
       <c r="L337" t="s">
         <v>50</v>
@@ -26818,7 +26818,7 @@
         <v>128</v>
       </c>
       <c r="K338" t="n">
-        <v>0.025111538461536</v>
+        <v>2.5111538461536</v>
       </c>
       <c r="L338" t="s">
         <v>50</v>
@@ -27665,7 +27665,7 @@
         <v>49</v>
       </c>
       <c r="K349" t="n">
-        <v>0.884891849806451</v>
+        <v>88.4891849806451</v>
       </c>
       <c r="L349" t="s">
         <v>50</v>
@@ -27742,7 +27742,7 @@
         <v>55</v>
       </c>
       <c r="K350" t="n">
-        <v>2.41934179830092</v>
+        <v>241.934179830092</v>
       </c>
       <c r="L350" t="s">
         <v>50</v>
@@ -27819,7 +27819,7 @@
         <v>58</v>
       </c>
       <c r="K351" t="n">
-        <v>8.92805062344325</v>
+        <v>892.805062344325</v>
       </c>
       <c r="L351" t="s">
         <v>50</v>
@@ -27896,7 +27896,7 @@
         <v>61</v>
       </c>
       <c r="K352" t="n">
-        <v>7.46338125985779</v>
+        <v>746.33812598578</v>
       </c>
       <c r="L352" t="s">
         <v>50</v>
@@ -27973,7 +27973,7 @@
         <v>64</v>
       </c>
       <c r="K353" t="n">
-        <v>19.1436581215066</v>
+        <v>1914.36581215066</v>
       </c>
       <c r="L353" t="s">
         <v>50</v>
@@ -28050,7 +28050,7 @@
         <v>67</v>
       </c>
       <c r="K354" t="n">
-        <v>16.5729645572602</v>
+        <v>1657.29645572602</v>
       </c>
       <c r="L354" t="s">
         <v>50</v>
@@ -28127,7 +28127,7 @@
         <v>70</v>
       </c>
       <c r="K355" t="n">
-        <v>4.65919425072088</v>
+        <v>465.919425072088</v>
       </c>
       <c r="L355" t="s">
         <v>50</v>
@@ -28204,7 +28204,7 @@
         <v>74</v>
       </c>
       <c r="K356" t="n">
-        <v>0.143017674418607</v>
+        <v>14.3017674418607</v>
       </c>
       <c r="L356" t="s">
         <v>50</v>
@@ -28281,7 +28281,7 @@
         <v>77</v>
       </c>
       <c r="K357" t="n">
-        <v>0.0513969767441869</v>
+        <v>5.13969767441869</v>
       </c>
       <c r="L357" t="s">
         <v>50</v>
@@ -28358,7 +28358,7 @@
         <v>80</v>
       </c>
       <c r="K358" t="n">
-        <v>0.0737434883720942</v>
+        <v>7.37434883720942</v>
       </c>
       <c r="L358" t="s">
         <v>50</v>
@@ -28435,7 +28435,7 @@
         <v>132</v>
       </c>
       <c r="K359" t="n">
-        <v>0.0223465116279073</v>
+        <v>2.23465116279073</v>
       </c>
       <c r="L359" t="s">
         <v>50</v>
@@ -28512,7 +28512,7 @@
         <v>135</v>
       </c>
       <c r="K360" t="n">
-        <v>0.0245811627906981</v>
+        <v>2.45811627906981</v>
       </c>
       <c r="L360" t="s">
         <v>50</v>
@@ -28589,7 +28589,7 @@
         <v>128</v>
       </c>
       <c r="K361" t="n">
-        <v>0.00223465116279073</v>
+        <v>0.223465116279073</v>
       </c>
       <c r="L361" t="s">
         <v>50</v>
@@ -29590,7 +29590,7 @@
         <v>49</v>
       </c>
       <c r="K374" t="n">
-        <v>0.456889827277793</v>
+        <v>45.6889827277793</v>
       </c>
       <c r="L374" t="s">
         <v>50</v>
@@ -29667,7 +29667,7 @@
         <v>55</v>
       </c>
       <c r="K375" t="n">
-        <v>1.25203366470191</v>
+        <v>125.203366470191</v>
       </c>
       <c r="L375" t="s">
         <v>50</v>
@@ -29744,7 +29744,7 @@
         <v>58</v>
       </c>
       <c r="K376" t="n">
-        <v>3.94957332629542</v>
+        <v>394.957332629542</v>
       </c>
       <c r="L376" t="s">
         <v>50</v>
@@ -29821,7 +29821,7 @@
         <v>61</v>
       </c>
       <c r="K377" t="n">
-        <v>2.96303334213073</v>
+        <v>296.303334213073</v>
       </c>
       <c r="L377" t="s">
         <v>50</v>
@@ -29898,7 +29898,7 @@
         <v>64</v>
       </c>
       <c r="K378" t="n">
-        <v>6.14628310020234</v>
+        <v>614.628310020234</v>
       </c>
       <c r="L378" t="s">
         <v>50</v>
@@ -29975,7 +29975,7 @@
         <v>67</v>
       </c>
       <c r="K379" t="n">
-        <v>5.74383155919181</v>
+        <v>574.383155919181</v>
       </c>
       <c r="L379" t="s">
         <v>50</v>
@@ -30052,7 +30052,7 @@
         <v>70</v>
       </c>
       <c r="K380" t="n">
-        <v>1.81194686372834</v>
+        <v>181.194686372834</v>
       </c>
       <c r="L380" t="s">
         <v>50</v>
@@ -30129,7 +30129,7 @@
         <v>74</v>
       </c>
       <c r="K381" t="n">
-        <v>0.0765432098765432</v>
+        <v>7.65432098765432</v>
       </c>
       <c r="L381" t="s">
         <v>50</v>
@@ -30206,7 +30206,7 @@
         <v>77</v>
       </c>
       <c r="K382" t="n">
-        <v>0.0197530864197531</v>
+        <v>1.97530864197531</v>
       </c>
       <c r="L382" t="s">
         <v>50</v>
@@ -30283,7 +30283,7 @@
         <v>80</v>
       </c>
       <c r="K383" t="n">
-        <v>0.0518518518518519</v>
+        <v>5.18518518518519</v>
       </c>
       <c r="L383" t="s">
         <v>50</v>
@@ -30360,7 +30360,7 @@
         <v>132</v>
       </c>
       <c r="K384" t="n">
-        <v>0.0119753086419753</v>
+        <v>1.19753086419753</v>
       </c>
       <c r="L384" t="s">
         <v>50</v>
@@ -30437,7 +30437,7 @@
         <v>135</v>
       </c>
       <c r="K385" t="n">
-        <v>0.0107407407407407</v>
+        <v>1.07407407407407</v>
       </c>
       <c r="L385" t="s">
         <v>50</v>
@@ -30514,7 +30514,7 @@
         <v>128</v>
       </c>
       <c r="K386" t="n">
-        <v>0.0288554587841999</v>
+        <v>2.88554587841999</v>
       </c>
       <c r="L386" t="s">
         <v>50</v>

</xml_diff>